<commit_message>
created google candidates models
started calling Google API from code and getting response.
</commit_message>
<xml_diff>
--- a/assets/test_file_2020_11_26_copy.xlsx
+++ b/assets/test_file_2020_11_26_copy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jared\source\repos\avtopia\data_sync_desktop\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE3C0C7C-CF7E-435C-9456-081318714A27}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A063D07B-BE6C-4E7D-84E3-B60776E97E9F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,9 +16,9 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AT$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AT$263</definedName>
   </definedNames>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2497" uniqueCount="1637">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2499" uniqueCount="1639">
   <si>
     <t>Account: Account Name</t>
   </si>
@@ -3420,9 +3420,6 @@
     <t>55347</t>
   </si>
   <si>
-    <t>(952) 851-0631 ext 322</t>
-  </si>
-  <si>
     <t>http://www.thunderbirdaviation.com</t>
   </si>
   <si>
@@ -3840,9 +3837,6 @@
     <t>74115-1400</t>
   </si>
   <si>
-    <t>(918) 836-7345, x254</t>
-  </si>
-  <si>
     <t>http://www.unitedstatesaviation.com</t>
   </si>
   <si>
@@ -4132,9 +4126,6 @@
   </si>
   <si>
     <t>11735-3324</t>
-  </si>
-  <si>
-    <t>(631) 756-5500, x126</t>
   </si>
   <si>
     <t>http://www.ventura.aero</t>
@@ -5010,6 +5001,21 @@
   </si>
   <si>
     <t>Google:SyncByAddress</t>
+  </si>
+  <si>
+    <t>(284) 495-1298</t>
+  </si>
+  <si>
+    <t>http://www.platinumbviservices.com/</t>
+  </si>
+  <si>
+    <t>(952) 851-0631</t>
+  </si>
+  <si>
+    <t>(918) 836-7345</t>
+  </si>
+  <si>
+    <t>(631) 756-5500</t>
   </si>
 </sst>
 </file>
@@ -5128,7 +5134,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5172,6 +5178,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -5525,7 +5532,7 @@
     <col min="10" max="10" width="5.125" style="3" customWidth="1"/>
     <col min="11" max="11" width="11.5" style="3" customWidth="1"/>
     <col min="12" max="12" width="12.875" style="3" customWidth="1"/>
-    <col min="13" max="13" width="13.75" style="3" customWidth="1"/>
+    <col min="13" max="13" width="23.5" style="3" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="55.125" style="3" bestFit="1" customWidth="1"/>
     <col min="15" max="21" width="12.125" style="4" bestFit="1" customWidth="1"/>
     <col min="22" max="23" width="12.125" style="3" bestFit="1" customWidth="1"/>
@@ -5537,10 +5544,10 @@
   <sheetData>
     <row r="1" spans="1:46">
       <c r="A1" s="18" t="s">
-        <v>1629</v>
+        <v>1626</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>1630</v>
+        <v>1627</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -5669,10 +5676,10 @@
         <v>41</v>
       </c>
       <c r="AS1" s="3" t="s">
-        <v>1635</v>
+        <v>1632</v>
       </c>
       <c r="AT1" s="3" t="s">
-        <v>1636</v>
+        <v>1633</v>
       </c>
     </row>
     <row r="2" spans="1:46" ht="15.75" customHeight="1">
@@ -5680,7 +5687,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>1631</v>
+        <v>1628</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>42</v>
@@ -5713,7 +5720,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>1632</v>
+        <v>1629</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>50</v>
@@ -5749,7 +5756,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>1633</v>
+        <v>1630</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>57</v>
@@ -5784,7 +5791,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>1634</v>
+        <v>1631</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>64</v>
@@ -6088,26 +6095,31 @@
       </c>
     </row>
     <row r="14" spans="1:46">
-      <c r="A14" s="3">
+      <c r="A14" s="23">
         <v>13</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="B14" s="23"/>
+      <c r="C14" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="G14" s="5" t="s">
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="I14" s="5" t="s">
+      <c r="H14" s="23"/>
+      <c r="I14" s="22" t="s">
         <v>132</v>
       </c>
-      <c r="J14" s="5" t="s">
+      <c r="J14" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="K14" s="5" t="s">
+      <c r="K14" s="22" t="s">
         <v>134</v>
       </c>
       <c r="L14" s="22" t="s">
-        <v>135</v>
+        <v>47</v>
       </c>
       <c r="M14" s="22" t="s">
         <v>136</v>
@@ -6120,29 +6132,38 @@
       </c>
     </row>
     <row r="15" spans="1:46">
-      <c r="A15" s="3">
+      <c r="A15" s="23">
         <v>14</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="B15" s="23"/>
+      <c r="C15" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="G15" s="5" t="s">
+      <c r="D15" s="23"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="I15" s="5" t="s">
+      <c r="H15" s="23"/>
+      <c r="I15" s="22" t="s">
         <v>141</v>
       </c>
-      <c r="J15" s="5" t="s">
+      <c r="J15" s="22" t="s">
         <v>142</v>
       </c>
-      <c r="K15" s="5" t="s">
+      <c r="K15" s="22" t="s">
         <v>143</v>
       </c>
-      <c r="L15" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M15" s="5"/>
-      <c r="N15" s="5"/>
+      <c r="L15" s="22" t="s">
+        <v>135</v>
+      </c>
+      <c r="M15" s="22" t="s">
+        <v>1634</v>
+      </c>
+      <c r="N15" s="5" t="s">
+        <v>1635</v>
+      </c>
       <c r="O15" s="4" t="s">
         <v>78</v>
       </c>
@@ -11722,10 +11743,10 @@
         <v>47</v>
       </c>
       <c r="M177" s="5" t="s">
+        <v>1636</v>
+      </c>
+      <c r="N177" s="5" t="s">
         <v>1127</v>
-      </c>
-      <c r="N177" s="5" t="s">
-        <v>1128</v>
       </c>
       <c r="O177" s="4" t="s">
         <v>78</v>
@@ -11745,31 +11766,31 @@
         <v>177</v>
       </c>
       <c r="C178" s="5" t="s">
+        <v>1128</v>
+      </c>
+      <c r="G178" s="5" t="s">
         <v>1129</v>
       </c>
-      <c r="G178" s="5" t="s">
+      <c r="H178" s="3" t="s">
         <v>1130</v>
       </c>
-      <c r="H178" s="3" t="s">
+      <c r="I178" s="5" t="s">
         <v>1131</v>
-      </c>
-      <c r="I178" s="5" t="s">
-        <v>1132</v>
       </c>
       <c r="J178" s="5" t="s">
         <v>226</v>
       </c>
       <c r="K178" s="5" t="s">
+        <v>1132</v>
+      </c>
+      <c r="L178" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M178" s="5" t="s">
         <v>1133</v>
       </c>
-      <c r="L178" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M178" s="5" t="s">
+      <c r="N178" s="5" t="s">
         <v>1134</v>
-      </c>
-      <c r="N178" s="5" t="s">
-        <v>1135</v>
       </c>
       <c r="O178" s="4" t="s">
         <v>78</v>
@@ -11789,25 +11810,25 @@
         <v>178</v>
       </c>
       <c r="C179" s="5" t="s">
+        <v>1135</v>
+      </c>
+      <c r="G179" s="5" t="s">
         <v>1136</v>
       </c>
-      <c r="G179" s="5" t="s">
+      <c r="I179" s="5" t="s">
         <v>1137</v>
-      </c>
-      <c r="I179" s="5" t="s">
-        <v>1138</v>
       </c>
       <c r="J179" s="5" t="s">
         <v>148</v>
       </c>
       <c r="K179" s="5" t="s">
+        <v>1138</v>
+      </c>
+      <c r="L179" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M179" s="5" t="s">
         <v>1139</v>
-      </c>
-      <c r="L179" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M179" s="5" t="s">
-        <v>1140</v>
       </c>
       <c r="N179" s="5"/>
       <c r="O179" s="4" t="s">
@@ -11819,25 +11840,25 @@
         <v>179</v>
       </c>
       <c r="C180" s="5" t="s">
+        <v>1140</v>
+      </c>
+      <c r="G180" s="5" t="s">
         <v>1141</v>
       </c>
-      <c r="G180" s="5" t="s">
+      <c r="I180" s="5" t="s">
         <v>1142</v>
       </c>
-      <c r="I180" s="5" t="s">
+      <c r="J180" s="5" t="s">
         <v>1143</v>
       </c>
-      <c r="J180" s="5" t="s">
+      <c r="K180" s="5" t="s">
         <v>1144</v>
       </c>
-      <c r="K180" s="5" t="s">
+      <c r="L180" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M180" s="5" t="s">
         <v>1145</v>
-      </c>
-      <c r="L180" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M180" s="5" t="s">
-        <v>1146</v>
       </c>
       <c r="N180" s="5"/>
       <c r="O180" s="4" t="s">
@@ -11849,25 +11870,25 @@
         <v>180</v>
       </c>
       <c r="C181" s="5" t="s">
+        <v>1146</v>
+      </c>
+      <c r="G181" s="5" t="s">
         <v>1147</v>
       </c>
-      <c r="G181" s="5" t="s">
+      <c r="I181" s="5" t="s">
         <v>1148</v>
-      </c>
-      <c r="I181" s="5" t="s">
-        <v>1149</v>
       </c>
       <c r="J181" s="5" t="s">
         <v>148</v>
       </c>
       <c r="K181" s="5" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L181" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M181" s="5" t="s">
         <v>1150</v>
-      </c>
-      <c r="L181" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M181" s="5" t="s">
-        <v>1151</v>
       </c>
       <c r="N181" s="5"/>
       <c r="O181" s="4" t="s">
@@ -11879,31 +11900,31 @@
         <v>181</v>
       </c>
       <c r="C182" s="5" t="s">
+        <v>1151</v>
+      </c>
+      <c r="G182" s="5" t="s">
         <v>1152</v>
       </c>
-      <c r="G182" s="5" t="s">
+      <c r="H182" s="3" t="s">
         <v>1153</v>
       </c>
-      <c r="H182" s="3" t="s">
+      <c r="I182" s="5" t="s">
         <v>1154</v>
-      </c>
-      <c r="I182" s="5" t="s">
-        <v>1155</v>
       </c>
       <c r="J182" s="5" t="s">
         <v>226</v>
       </c>
       <c r="K182" s="5" t="s">
+        <v>1155</v>
+      </c>
+      <c r="L182" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M182" s="5" t="s">
         <v>1156</v>
       </c>
-      <c r="L182" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M182" s="5" t="s">
+      <c r="N182" s="5" t="s">
         <v>1157</v>
-      </c>
-      <c r="N182" s="5" t="s">
-        <v>1158</v>
       </c>
       <c r="O182" s="4" t="s">
         <v>78</v>
@@ -11914,32 +11935,32 @@
         <v>182</v>
       </c>
       <c r="C183" s="5" t="s">
+        <v>1158</v>
+      </c>
+      <c r="G183" s="5" t="s">
         <v>1159</v>
       </c>
-      <c r="G183" s="5" t="s">
+      <c r="H183" s="3" t="s">
         <v>1160</v>
       </c>
-      <c r="H183" s="3" t="s">
+      <c r="I183" s="5" t="s">
         <v>1161</v>
-      </c>
-      <c r="I183" s="5" t="s">
-        <v>1162</v>
       </c>
       <c r="J183" s="5" t="s">
         <v>512</v>
       </c>
       <c r="K183" s="5" t="s">
+        <v>1162</v>
+      </c>
+      <c r="L183" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M183" s="5" t="s">
         <v>1163</v>
-      </c>
-      <c r="L183" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M183" s="5" t="s">
-        <v>1164</v>
       </c>
       <c r="N183" s="5"/>
       <c r="O183" s="4" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="184" spans="1:21">
@@ -11947,25 +11968,25 @@
         <v>183</v>
       </c>
       <c r="C184" s="5" t="s">
+        <v>1165</v>
+      </c>
+      <c r="G184" s="5" t="s">
         <v>1166</v>
       </c>
-      <c r="G184" s="5" t="s">
+      <c r="I184" s="5" t="s">
         <v>1167</v>
-      </c>
-      <c r="I184" s="5" t="s">
-        <v>1168</v>
       </c>
       <c r="J184" s="5" t="s">
         <v>430</v>
       </c>
       <c r="K184" s="5" t="s">
+        <v>1168</v>
+      </c>
+      <c r="L184" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M184" s="5" t="s">
         <v>1169</v>
-      </c>
-      <c r="L184" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M184" s="5" t="s">
-        <v>1170</v>
       </c>
       <c r="N184" s="5"/>
       <c r="O184" s="4" t="s">
@@ -11977,28 +11998,28 @@
         <v>184</v>
       </c>
       <c r="C185" s="5" t="s">
+        <v>1170</v>
+      </c>
+      <c r="G185" s="5" t="s">
         <v>1171</v>
       </c>
-      <c r="G185" s="5" t="s">
+      <c r="I185" s="5" t="s">
         <v>1172</v>
-      </c>
-      <c r="I185" s="5" t="s">
-        <v>1173</v>
       </c>
       <c r="J185" s="5" t="s">
         <v>430</v>
       </c>
       <c r="K185" s="5" t="s">
+        <v>1173</v>
+      </c>
+      <c r="L185" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M185" s="5" t="s">
         <v>1174</v>
       </c>
-      <c r="L185" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M185" s="5" t="s">
+      <c r="N185" s="5" t="s">
         <v>1175</v>
-      </c>
-      <c r="N185" s="5" t="s">
-        <v>1176</v>
       </c>
       <c r="O185" s="4" t="s">
         <v>112</v>
@@ -12012,25 +12033,25 @@
         <v>185</v>
       </c>
       <c r="C186" s="5" t="s">
+        <v>1176</v>
+      </c>
+      <c r="G186" s="5" t="s">
         <v>1177</v>
       </c>
-      <c r="G186" s="5" t="s">
+      <c r="I186" s="5" t="s">
         <v>1178</v>
-      </c>
-      <c r="I186" s="5" t="s">
-        <v>1179</v>
       </c>
       <c r="J186" s="5" t="s">
         <v>54</v>
       </c>
       <c r="K186" s="5" t="s">
+        <v>1179</v>
+      </c>
+      <c r="L186" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M186" s="5" t="s">
         <v>1180</v>
-      </c>
-      <c r="L186" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M186" s="5" t="s">
-        <v>1181</v>
       </c>
       <c r="N186" s="5"/>
       <c r="O186" s="4" t="s">
@@ -12046,10 +12067,10 @@
       </c>
       <c r="B187" s="3"/>
       <c r="C187" s="7" t="s">
+        <v>1181</v>
+      </c>
+      <c r="G187" s="7" t="s">
         <v>1182</v>
-      </c>
-      <c r="G187" s="7" t="s">
-        <v>1183</v>
       </c>
       <c r="I187" s="7" t="s">
         <v>679</v>
@@ -12058,19 +12079,19 @@
         <v>299</v>
       </c>
       <c r="K187" s="7" t="s">
+        <v>1183</v>
+      </c>
+      <c r="L187" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="M187" s="7" t="s">
         <v>1184</v>
       </c>
-      <c r="L187" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="M187" s="7" t="s">
+      <c r="N187" s="7" t="s">
         <v>1185</v>
       </c>
-      <c r="N187" s="7" t="s">
+      <c r="O187" s="10" t="s">
         <v>1186</v>
-      </c>
-      <c r="O187" s="10" t="s">
-        <v>1187</v>
       </c>
       <c r="P187" s="16"/>
       <c r="Q187" s="10"/>
@@ -12084,28 +12105,28 @@
         <v>187</v>
       </c>
       <c r="C188" s="5" t="s">
+        <v>1187</v>
+      </c>
+      <c r="G188" s="5" t="s">
         <v>1188</v>
       </c>
-      <c r="G188" s="5" t="s">
+      <c r="I188" s="5" t="s">
         <v>1189</v>
       </c>
-      <c r="I188" s="5" t="s">
+      <c r="J188" s="5" t="s">
         <v>1190</v>
       </c>
-      <c r="J188" s="5" t="s">
+      <c r="K188" s="5" t="s">
         <v>1191</v>
       </c>
-      <c r="K188" s="5" t="s">
+      <c r="L188" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M188" s="5" t="s">
         <v>1192</v>
       </c>
-      <c r="L188" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M188" s="5" t="s">
+      <c r="N188" s="5" t="s">
         <v>1193</v>
-      </c>
-      <c r="N188" s="5" t="s">
-        <v>1194</v>
       </c>
       <c r="O188" s="4" t="s">
         <v>78</v>
@@ -12122,28 +12143,28 @@
         <v>188</v>
       </c>
       <c r="C189" s="5" t="s">
+        <v>1194</v>
+      </c>
+      <c r="G189" s="5" t="s">
         <v>1195</v>
       </c>
-      <c r="G189" s="5" t="s">
+      <c r="I189" s="5" t="s">
         <v>1196</v>
-      </c>
-      <c r="I189" s="5" t="s">
-        <v>1197</v>
       </c>
       <c r="J189" s="5" t="s">
         <v>783</v>
       </c>
       <c r="K189" s="5" t="s">
+        <v>1197</v>
+      </c>
+      <c r="L189" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M189" s="5" t="s">
         <v>1198</v>
       </c>
-      <c r="L189" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M189" s="5" t="s">
+      <c r="N189" s="5" t="s">
         <v>1199</v>
-      </c>
-      <c r="N189" s="5" t="s">
-        <v>1200</v>
       </c>
       <c r="O189" s="4" t="s">
         <v>170</v>
@@ -12154,28 +12175,28 @@
         <v>189</v>
       </c>
       <c r="C190" s="5" t="s">
+        <v>1200</v>
+      </c>
+      <c r="G190" s="5" t="s">
         <v>1201</v>
       </c>
-      <c r="G190" s="5" t="s">
+      <c r="I190" s="5" t="s">
         <v>1202</v>
-      </c>
-      <c r="I190" s="5" t="s">
-        <v>1203</v>
       </c>
       <c r="J190" s="5" t="s">
         <v>54</v>
       </c>
       <c r="K190" s="5" t="s">
+        <v>1203</v>
+      </c>
+      <c r="L190" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M190" s="5" t="s">
         <v>1204</v>
       </c>
-      <c r="L190" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M190" s="5" t="s">
+      <c r="N190" s="5" t="s">
         <v>1205</v>
-      </c>
-      <c r="N190" s="5" t="s">
-        <v>1206</v>
       </c>
       <c r="O190" s="4" t="s">
         <v>170</v>
@@ -12186,28 +12207,28 @@
         <v>190</v>
       </c>
       <c r="C191" s="5" t="s">
+        <v>1206</v>
+      </c>
+      <c r="G191" s="5" t="s">
         <v>1207</v>
       </c>
-      <c r="G191" s="5" t="s">
+      <c r="I191" s="5" t="s">
         <v>1208</v>
-      </c>
-      <c r="I191" s="5" t="s">
-        <v>1209</v>
       </c>
       <c r="J191" s="5" t="s">
         <v>627</v>
       </c>
       <c r="K191" s="5" t="s">
+        <v>1209</v>
+      </c>
+      <c r="L191" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M191" s="5" t="s">
         <v>1210</v>
       </c>
-      <c r="L191" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M191" s="5" t="s">
+      <c r="N191" s="5" t="s">
         <v>1211</v>
-      </c>
-      <c r="N191" s="5" t="s">
-        <v>1212</v>
       </c>
       <c r="O191" s="4" t="s">
         <v>78</v>
@@ -12218,28 +12239,28 @@
         <v>191</v>
       </c>
       <c r="C192" s="5" t="s">
+        <v>1212</v>
+      </c>
+      <c r="G192" s="5" t="s">
         <v>1213</v>
       </c>
-      <c r="G192" s="5" t="s">
+      <c r="I192" s="5" t="s">
         <v>1214</v>
-      </c>
-      <c r="I192" s="5" t="s">
-        <v>1215</v>
       </c>
       <c r="J192" s="5" t="s">
         <v>180</v>
       </c>
       <c r="K192" s="5" t="s">
+        <v>1215</v>
+      </c>
+      <c r="L192" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M192" s="5" t="s">
         <v>1216</v>
       </c>
-      <c r="L192" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M192" s="5" t="s">
+      <c r="N192" s="5" t="s">
         <v>1217</v>
-      </c>
-      <c r="N192" s="5" t="s">
-        <v>1218</v>
       </c>
       <c r="O192" s="4" t="s">
         <v>78</v>
@@ -12250,28 +12271,28 @@
         <v>192</v>
       </c>
       <c r="C193" s="5" t="s">
+        <v>1218</v>
+      </c>
+      <c r="G193" s="5" t="s">
         <v>1219</v>
       </c>
-      <c r="G193" s="5" t="s">
+      <c r="I193" s="5" t="s">
         <v>1220</v>
-      </c>
-      <c r="I193" s="5" t="s">
-        <v>1221</v>
       </c>
       <c r="J193" s="5" t="s">
         <v>834</v>
       </c>
       <c r="K193" s="5" t="s">
+        <v>1221</v>
+      </c>
+      <c r="L193" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M193" s="5" t="s">
         <v>1222</v>
       </c>
-      <c r="L193" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M193" s="5" t="s">
+      <c r="N193" s="5" t="s">
         <v>1223</v>
-      </c>
-      <c r="N193" s="5" t="s">
-        <v>1224</v>
       </c>
       <c r="O193" s="4" t="s">
         <v>78</v>
@@ -12288,28 +12309,28 @@
         <v>193</v>
       </c>
       <c r="C194" s="5" t="s">
+        <v>1224</v>
+      </c>
+      <c r="G194" s="5" t="s">
         <v>1225</v>
       </c>
-      <c r="G194" s="5" t="s">
+      <c r="I194" s="5" t="s">
         <v>1226</v>
-      </c>
-      <c r="I194" s="5" t="s">
-        <v>1227</v>
       </c>
       <c r="J194" s="5" t="s">
         <v>212</v>
       </c>
       <c r="K194" s="5" t="s">
+        <v>1227</v>
+      </c>
+      <c r="L194" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M194" s="5" t="s">
         <v>1228</v>
       </c>
-      <c r="L194" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M194" s="5" t="s">
+      <c r="N194" s="5" t="s">
         <v>1229</v>
-      </c>
-      <c r="N194" s="5" t="s">
-        <v>1230</v>
       </c>
       <c r="O194" s="4" t="s">
         <v>49</v>
@@ -12320,28 +12341,28 @@
         <v>194</v>
       </c>
       <c r="C195" s="5" t="s">
+        <v>1230</v>
+      </c>
+      <c r="G195" s="5" t="s">
         <v>1231</v>
       </c>
-      <c r="G195" s="5" t="s">
+      <c r="I195" s="5" t="s">
         <v>1232</v>
-      </c>
-      <c r="I195" s="5" t="s">
-        <v>1233</v>
       </c>
       <c r="J195" s="5" t="s">
         <v>293</v>
       </c>
       <c r="K195" s="5" t="s">
+        <v>1233</v>
+      </c>
+      <c r="L195" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M195" s="5" t="s">
         <v>1234</v>
       </c>
-      <c r="L195" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M195" s="5" t="s">
+      <c r="N195" s="5" t="s">
         <v>1235</v>
-      </c>
-      <c r="N195" s="5" t="s">
-        <v>1236</v>
       </c>
       <c r="O195" s="4" t="s">
         <v>170</v>
@@ -12352,31 +12373,31 @@
         <v>195</v>
       </c>
       <c r="C196" s="5" t="s">
+        <v>1236</v>
+      </c>
+      <c r="G196" s="5" t="s">
         <v>1237</v>
       </c>
-      <c r="G196" s="5" t="s">
+      <c r="H196" s="3" t="s">
         <v>1238</v>
       </c>
-      <c r="H196" s="3" t="s">
+      <c r="I196" s="5" t="s">
         <v>1239</v>
-      </c>
-      <c r="I196" s="5" t="s">
-        <v>1240</v>
       </c>
       <c r="J196" s="5" t="s">
         <v>119</v>
       </c>
       <c r="K196" s="5" t="s">
+        <v>1240</v>
+      </c>
+      <c r="L196" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M196" s="5" t="s">
         <v>1241</v>
       </c>
-      <c r="L196" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M196" s="5" t="s">
+      <c r="N196" s="5" t="s">
         <v>1242</v>
-      </c>
-      <c r="N196" s="5" t="s">
-        <v>1243</v>
       </c>
       <c r="O196" s="4" t="s">
         <v>78</v>
@@ -12387,28 +12408,28 @@
         <v>196</v>
       </c>
       <c r="C197" s="5" t="s">
+        <v>1243</v>
+      </c>
+      <c r="G197" s="5" t="s">
         <v>1244</v>
       </c>
-      <c r="G197" s="5" t="s">
+      <c r="I197" s="5" t="s">
         <v>1245</v>
       </c>
-      <c r="I197" s="5" t="s">
+      <c r="J197" s="5" t="s">
         <v>1246</v>
       </c>
-      <c r="J197" s="5" t="s">
+      <c r="K197" s="5" t="s">
         <v>1247</v>
       </c>
-      <c r="K197" s="5" t="s">
+      <c r="L197" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M197" s="5" t="s">
         <v>1248</v>
       </c>
-      <c r="L197" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M197" s="5" t="s">
+      <c r="N197" s="5" t="s">
         <v>1249</v>
-      </c>
-      <c r="N197" s="5" t="s">
-        <v>1250</v>
       </c>
       <c r="O197" s="4" t="s">
         <v>78</v>
@@ -12419,10 +12440,10 @@
         <v>197</v>
       </c>
       <c r="C198" s="5" t="s">
+        <v>1250</v>
+      </c>
+      <c r="G198" s="5" t="s">
         <v>1251</v>
-      </c>
-      <c r="G198" s="5" t="s">
-        <v>1252</v>
       </c>
       <c r="I198" s="5" t="s">
         <v>825</v>
@@ -12431,19 +12452,19 @@
         <v>60</v>
       </c>
       <c r="K198" s="5" t="s">
+        <v>1252</v>
+      </c>
+      <c r="L198" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M198" s="5" t="s">
         <v>1253</v>
       </c>
-      <c r="L198" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M198" s="5" t="s">
+      <c r="N198" s="5" t="s">
         <v>1254</v>
       </c>
-      <c r="N198" s="5" t="s">
+      <c r="O198" s="4" t="s">
         <v>1255</v>
-      </c>
-      <c r="O198" s="4" t="s">
-        <v>1256</v>
       </c>
     </row>
     <row r="199" spans="1:19">
@@ -12451,28 +12472,28 @@
         <v>198</v>
       </c>
       <c r="C199" s="5" t="s">
+        <v>1256</v>
+      </c>
+      <c r="G199" s="5" t="s">
         <v>1257</v>
       </c>
-      <c r="G199" s="5" t="s">
+      <c r="I199" s="5" t="s">
         <v>1258</v>
       </c>
-      <c r="I199" s="5" t="s">
+      <c r="J199" s="5" t="s">
+        <v>1190</v>
+      </c>
+      <c r="K199" s="5" t="s">
         <v>1259</v>
       </c>
-      <c r="J199" s="5" t="s">
-        <v>1191</v>
-      </c>
-      <c r="K199" s="5" t="s">
+      <c r="L199" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M199" s="5" t="s">
         <v>1260</v>
       </c>
-      <c r="L199" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M199" s="5" t="s">
+      <c r="N199" s="5" t="s">
         <v>1261</v>
-      </c>
-      <c r="N199" s="5" t="s">
-        <v>1262</v>
       </c>
       <c r="O199" s="4" t="s">
         <v>78</v>
@@ -12492,28 +12513,28 @@
         <v>199</v>
       </c>
       <c r="C200" s="5" t="s">
+        <v>1262</v>
+      </c>
+      <c r="G200" s="5" t="s">
         <v>1263</v>
       </c>
-      <c r="G200" s="5" t="s">
+      <c r="I200" s="5" t="s">
         <v>1264</v>
-      </c>
-      <c r="I200" s="5" t="s">
-        <v>1265</v>
       </c>
       <c r="J200" s="5" t="s">
         <v>100</v>
       </c>
       <c r="K200" s="5" t="s">
+        <v>1265</v>
+      </c>
+      <c r="L200" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M200" s="5" t="s">
+        <v>1637</v>
+      </c>
+      <c r="N200" s="5" t="s">
         <v>1266</v>
-      </c>
-      <c r="L200" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M200" s="5" t="s">
-        <v>1267</v>
-      </c>
-      <c r="N200" s="5" t="s">
-        <v>1268</v>
       </c>
       <c r="O200" s="4" t="s">
         <v>78</v>
@@ -12522,7 +12543,7 @@
         <v>112</v>
       </c>
       <c r="Q200" s="4" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="201" spans="1:19">
@@ -12530,10 +12551,10 @@
         <v>200</v>
       </c>
       <c r="C201" s="5" t="s">
-        <v>1270</v>
+        <v>1268</v>
       </c>
       <c r="G201" s="5" t="s">
-        <v>1271</v>
+        <v>1269</v>
       </c>
       <c r="I201" s="5" t="s">
         <v>856</v>
@@ -12542,28 +12563,28 @@
         <v>67</v>
       </c>
       <c r="K201" s="5" t="s">
+        <v>1270</v>
+      </c>
+      <c r="L201" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M201" s="5" t="s">
+        <v>1271</v>
+      </c>
+      <c r="N201" s="5" t="s">
         <v>1272</v>
       </c>
-      <c r="L201" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M201" s="5" t="s">
+      <c r="O201" s="4" t="s">
         <v>1273</v>
       </c>
-      <c r="N201" s="5" t="s">
+      <c r="P201" s="4" t="s">
         <v>1274</v>
-      </c>
-      <c r="O201" s="4" t="s">
-        <v>1275</v>
-      </c>
-      <c r="P201" s="4" t="s">
-        <v>1276</v>
       </c>
       <c r="Q201" s="4" t="s">
         <v>971</v>
       </c>
       <c r="R201" s="4" t="s">
-        <v>1277</v>
+        <v>1275</v>
       </c>
       <c r="S201" s="4" t="s">
         <v>1072</v>
@@ -12574,28 +12595,28 @@
         <v>201</v>
       </c>
       <c r="C202" s="5" t="s">
+        <v>1276</v>
+      </c>
+      <c r="G202" s="5" t="s">
+        <v>1277</v>
+      </c>
+      <c r="I202" s="5" t="s">
         <v>1278</v>
-      </c>
-      <c r="G202" s="5" t="s">
-        <v>1279</v>
-      </c>
-      <c r="I202" s="5" t="s">
-        <v>1280</v>
       </c>
       <c r="J202" s="5" t="s">
         <v>54</v>
       </c>
       <c r="K202" s="5" t="s">
+        <v>1279</v>
+      </c>
+      <c r="L202" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M202" s="5" t="s">
+        <v>1280</v>
+      </c>
+      <c r="N202" s="5" t="s">
         <v>1281</v>
-      </c>
-      <c r="L202" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M202" s="5" t="s">
-        <v>1282</v>
-      </c>
-      <c r="N202" s="5" t="s">
-        <v>1283</v>
       </c>
       <c r="O202" s="4" t="s">
         <v>78</v>
@@ -12615,31 +12636,31 @@
         <v>202</v>
       </c>
       <c r="C203" s="5" t="s">
+        <v>1282</v>
+      </c>
+      <c r="G203" s="5" t="s">
+        <v>1283</v>
+      </c>
+      <c r="H203" s="3" t="s">
         <v>1284</v>
       </c>
-      <c r="G203" s="5" t="s">
+      <c r="I203" s="5" t="s">
         <v>1285</v>
       </c>
-      <c r="H203" s="3" t="s">
+      <c r="J203" s="5" t="s">
+        <v>1143</v>
+      </c>
+      <c r="K203" s="5" t="s">
         <v>1286</v>
       </c>
-      <c r="I203" s="5" t="s">
+      <c r="L203" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M203" s="5" t="s">
         <v>1287</v>
       </c>
-      <c r="J203" s="5" t="s">
-        <v>1144</v>
-      </c>
-      <c r="K203" s="5" t="s">
+      <c r="N203" s="5" t="s">
         <v>1288</v>
-      </c>
-      <c r="L203" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M203" s="5" t="s">
-        <v>1289</v>
-      </c>
-      <c r="N203" s="5" t="s">
-        <v>1290</v>
       </c>
       <c r="O203" s="4" t="s">
         <v>114</v>
@@ -12650,28 +12671,28 @@
         <v>203</v>
       </c>
       <c r="C204" s="5" t="s">
+        <v>1289</v>
+      </c>
+      <c r="G204" s="5" t="s">
+        <v>1290</v>
+      </c>
+      <c r="I204" s="5" t="s">
         <v>1291</v>
-      </c>
-      <c r="G204" s="5" t="s">
-        <v>1292</v>
-      </c>
-      <c r="I204" s="5" t="s">
-        <v>1293</v>
       </c>
       <c r="J204" s="5" t="s">
         <v>67</v>
       </c>
       <c r="K204" s="5" t="s">
+        <v>1292</v>
+      </c>
+      <c r="L204" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M204" s="5" t="s">
+        <v>1293</v>
+      </c>
+      <c r="N204" s="5" t="s">
         <v>1294</v>
-      </c>
-      <c r="L204" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M204" s="5" t="s">
-        <v>1295</v>
-      </c>
-      <c r="N204" s="5" t="s">
-        <v>1296</v>
       </c>
       <c r="O204" s="4" t="s">
         <v>78</v>
@@ -12682,28 +12703,28 @@
         <v>204</v>
       </c>
       <c r="C205" s="5" t="s">
+        <v>1295</v>
+      </c>
+      <c r="G205" s="5" t="s">
+        <v>1296</v>
+      </c>
+      <c r="I205" s="5" t="s">
         <v>1297</v>
-      </c>
-      <c r="G205" s="5" t="s">
-        <v>1298</v>
-      </c>
-      <c r="I205" s="5" t="s">
-        <v>1299</v>
       </c>
       <c r="J205" s="5" t="s">
         <v>54</v>
       </c>
       <c r="K205" s="5" t="s">
+        <v>1298</v>
+      </c>
+      <c r="L205" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M205" s="5" t="s">
+        <v>1299</v>
+      </c>
+      <c r="N205" s="5" t="s">
         <v>1300</v>
-      </c>
-      <c r="L205" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M205" s="5" t="s">
-        <v>1301</v>
-      </c>
-      <c r="N205" s="5" t="s">
-        <v>1302</v>
       </c>
       <c r="O205" s="4" t="s">
         <v>114</v>
@@ -12714,31 +12735,31 @@
         <v>205</v>
       </c>
       <c r="C206" s="5" t="s">
+        <v>1301</v>
+      </c>
+      <c r="G206" s="5" t="s">
+        <v>1302</v>
+      </c>
+      <c r="I206" s="5" t="s">
         <v>1303</v>
-      </c>
-      <c r="G206" s="5" t="s">
-        <v>1304</v>
-      </c>
-      <c r="I206" s="5" t="s">
-        <v>1305</v>
       </c>
       <c r="J206" s="5" t="s">
         <v>108</v>
       </c>
       <c r="K206" s="5" t="s">
+        <v>1304</v>
+      </c>
+      <c r="L206" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M206" s="5" t="s">
+        <v>1305</v>
+      </c>
+      <c r="N206" s="5" t="s">
         <v>1306</v>
       </c>
-      <c r="L206" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M206" s="5" t="s">
+      <c r="O206" s="4" t="s">
         <v>1307</v>
-      </c>
-      <c r="N206" s="5" t="s">
-        <v>1308</v>
-      </c>
-      <c r="O206" s="4" t="s">
-        <v>1309</v>
       </c>
     </row>
     <row r="207" spans="1:19">
@@ -12746,25 +12767,25 @@
         <v>206</v>
       </c>
       <c r="C207" s="5" t="s">
+        <v>1308</v>
+      </c>
+      <c r="G207" s="5" t="s">
+        <v>1309</v>
+      </c>
+      <c r="I207" s="5" t="s">
         <v>1310</v>
-      </c>
-      <c r="G207" s="5" t="s">
-        <v>1311</v>
-      </c>
-      <c r="I207" s="5" t="s">
-        <v>1312</v>
       </c>
       <c r="J207" s="5" t="s">
         <v>67</v>
       </c>
       <c r="K207" s="5" t="s">
-        <v>1313</v>
+        <v>1311</v>
       </c>
       <c r="L207" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M207" s="5" t="s">
-        <v>1314</v>
+        <v>1312</v>
       </c>
       <c r="N207" s="5"/>
       <c r="O207" s="4" t="s">
@@ -12776,25 +12797,25 @@
         <v>207</v>
       </c>
       <c r="C208" s="5" t="s">
+        <v>1313</v>
+      </c>
+      <c r="G208" s="5" t="s">
+        <v>1314</v>
+      </c>
+      <c r="I208" s="5" t="s">
         <v>1315</v>
-      </c>
-      <c r="G208" s="5" t="s">
-        <v>1316</v>
-      </c>
-      <c r="I208" s="5" t="s">
-        <v>1317</v>
       </c>
       <c r="J208" s="5" t="s">
         <v>212</v>
       </c>
       <c r="K208" s="5" t="s">
-        <v>1318</v>
+        <v>1316</v>
       </c>
       <c r="L208" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M208" s="5" t="s">
-        <v>1319</v>
+        <v>1317</v>
       </c>
       <c r="N208" s="5"/>
       <c r="O208" s="4" t="s">
@@ -12806,28 +12827,28 @@
         <v>208</v>
       </c>
       <c r="C209" s="5" t="s">
+        <v>1318</v>
+      </c>
+      <c r="G209" s="5" t="s">
+        <v>1319</v>
+      </c>
+      <c r="I209" s="5" t="s">
         <v>1320</v>
-      </c>
-      <c r="G209" s="5" t="s">
-        <v>1321</v>
-      </c>
-      <c r="I209" s="5" t="s">
-        <v>1322</v>
       </c>
       <c r="J209" s="5" t="s">
         <v>108</v>
       </c>
       <c r="K209" s="5" t="s">
+        <v>1321</v>
+      </c>
+      <c r="L209" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M209" s="5" t="s">
+        <v>1322</v>
+      </c>
+      <c r="N209" s="5" t="s">
         <v>1323</v>
-      </c>
-      <c r="L209" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M209" s="5" t="s">
-        <v>1324</v>
-      </c>
-      <c r="N209" s="5" t="s">
-        <v>1325</v>
       </c>
       <c r="O209" s="4" t="s">
         <v>78</v>
@@ -12838,28 +12859,28 @@
         <v>209</v>
       </c>
       <c r="C210" s="5" t="s">
+        <v>1324</v>
+      </c>
+      <c r="G210" s="5" t="s">
+        <v>1325</v>
+      </c>
+      <c r="I210" s="5" t="s">
         <v>1326</v>
       </c>
-      <c r="G210" s="5" t="s">
+      <c r="J210" s="5" t="s">
+        <v>1190</v>
+      </c>
+      <c r="K210" s="5" t="s">
         <v>1327</v>
       </c>
-      <c r="I210" s="5" t="s">
+      <c r="L210" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M210" s="5" t="s">
         <v>1328</v>
       </c>
-      <c r="J210" s="5" t="s">
-        <v>1191</v>
-      </c>
-      <c r="K210" s="5" t="s">
+      <c r="N210" s="5" t="s">
         <v>1329</v>
-      </c>
-      <c r="L210" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M210" s="5" t="s">
-        <v>1330</v>
-      </c>
-      <c r="N210" s="5" t="s">
-        <v>1331</v>
       </c>
       <c r="O210" s="4" t="s">
         <v>78</v>
@@ -12871,10 +12892,10 @@
       </c>
       <c r="B211" s="3"/>
       <c r="C211" s="7" t="s">
-        <v>1332</v>
+        <v>1330</v>
       </c>
       <c r="G211" s="12" t="s">
-        <v>1333</v>
+        <v>1331</v>
       </c>
       <c r="I211" s="12" t="s">
         <v>899</v>
@@ -12883,16 +12904,16 @@
         <v>299</v>
       </c>
       <c r="K211" s="12" t="s">
+        <v>1332</v>
+      </c>
+      <c r="L211" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="M211" s="12" t="s">
+        <v>1333</v>
+      </c>
+      <c r="N211" s="12" t="s">
         <v>1334</v>
-      </c>
-      <c r="L211" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="M211" s="12" t="s">
-        <v>1335</v>
-      </c>
-      <c r="N211" s="12" t="s">
-        <v>1336</v>
       </c>
       <c r="O211" s="10" t="s">
         <v>170</v>
@@ -12909,28 +12930,28 @@
         <v>211</v>
       </c>
       <c r="C212" s="5" t="s">
+        <v>1335</v>
+      </c>
+      <c r="G212" s="5" t="s">
+        <v>1336</v>
+      </c>
+      <c r="I212" s="5" t="s">
         <v>1337</v>
-      </c>
-      <c r="G212" s="5" t="s">
-        <v>1338</v>
-      </c>
-      <c r="I212" s="5" t="s">
-        <v>1339</v>
       </c>
       <c r="J212" s="5" t="s">
         <v>148</v>
       </c>
       <c r="K212" s="5" t="s">
+        <v>1338</v>
+      </c>
+      <c r="L212" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M212" s="5" t="s">
+        <v>1339</v>
+      </c>
+      <c r="N212" s="5" t="s">
         <v>1340</v>
-      </c>
-      <c r="L212" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M212" s="5" t="s">
-        <v>1341</v>
-      </c>
-      <c r="N212" s="5" t="s">
-        <v>1342</v>
       </c>
       <c r="O212" s="4" t="s">
         <v>115</v>
@@ -12941,28 +12962,28 @@
         <v>212</v>
       </c>
       <c r="C213" s="5" t="s">
+        <v>1341</v>
+      </c>
+      <c r="G213" s="5" t="s">
+        <v>1342</v>
+      </c>
+      <c r="I213" s="5" t="s">
         <v>1343</v>
-      </c>
-      <c r="G213" s="5" t="s">
-        <v>1344</v>
-      </c>
-      <c r="I213" s="5" t="s">
-        <v>1345</v>
       </c>
       <c r="J213" s="5" t="s">
         <v>75</v>
       </c>
       <c r="K213" s="5" t="s">
+        <v>1344</v>
+      </c>
+      <c r="L213" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M213" s="5" t="s">
+        <v>1345</v>
+      </c>
+      <c r="N213" s="5" t="s">
         <v>1346</v>
-      </c>
-      <c r="L213" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M213" s="5" t="s">
-        <v>1347</v>
-      </c>
-      <c r="N213" s="5" t="s">
-        <v>1348</v>
       </c>
       <c r="O213" s="4" t="s">
         <v>78</v>
@@ -12973,34 +12994,34 @@
         <v>213</v>
       </c>
       <c r="C214" s="5" t="s">
+        <v>1347</v>
+      </c>
+      <c r="D214" s="3" t="s">
+        <v>1348</v>
+      </c>
+      <c r="G214" s="5" t="s">
         <v>1349</v>
       </c>
-      <c r="D214" s="3" t="s">
+      <c r="I214" s="5" t="s">
         <v>1350</v>
-      </c>
-      <c r="G214" s="5" t="s">
-        <v>1351</v>
-      </c>
-      <c r="I214" s="5" t="s">
-        <v>1352</v>
       </c>
       <c r="J214" s="5" t="s">
         <v>274</v>
       </c>
       <c r="K214" s="5" t="s">
+        <v>1351</v>
+      </c>
+      <c r="L214" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M214" s="5" t="s">
+        <v>1352</v>
+      </c>
+      <c r="N214" s="5" t="s">
         <v>1353</v>
       </c>
-      <c r="L214" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M214" s="5" t="s">
+      <c r="O214" s="4" t="s">
         <v>1354</v>
-      </c>
-      <c r="N214" s="5" t="s">
-        <v>1355</v>
-      </c>
-      <c r="O214" s="4" t="s">
-        <v>1356</v>
       </c>
       <c r="P214" s="4" t="s">
         <v>78</v>
@@ -13020,10 +13041,10 @@
         <v>214</v>
       </c>
       <c r="C215" s="5" t="s">
-        <v>1357</v>
+        <v>1355</v>
       </c>
       <c r="G215" s="5" t="s">
-        <v>1358</v>
+        <v>1356</v>
       </c>
       <c r="I215" s="5" t="s">
         <v>205</v>
@@ -13032,16 +13053,16 @@
         <v>126</v>
       </c>
       <c r="K215" s="5" t="s">
+        <v>1357</v>
+      </c>
+      <c r="L215" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M215" s="5" t="s">
+        <v>1358</v>
+      </c>
+      <c r="N215" s="5" t="s">
         <v>1359</v>
-      </c>
-      <c r="L215" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M215" s="5" t="s">
-        <v>1360</v>
-      </c>
-      <c r="N215" s="5" t="s">
-        <v>1361</v>
       </c>
       <c r="O215" s="4" t="s">
         <v>112</v>
@@ -13052,10 +13073,10 @@
         <v>215</v>
       </c>
       <c r="C216" s="5" t="s">
-        <v>1362</v>
+        <v>1360</v>
       </c>
       <c r="G216" s="5" t="s">
-        <v>1363</v>
+        <v>1361</v>
       </c>
       <c r="I216" s="5" t="s">
         <v>1017</v>
@@ -13064,16 +13085,16 @@
         <v>219</v>
       </c>
       <c r="K216" s="5" t="s">
-        <v>1364</v>
+        <v>1362</v>
       </c>
       <c r="L216" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M216" s="5" t="s">
-        <v>1365</v>
+        <v>1638</v>
       </c>
       <c r="N216" s="5" t="s">
-        <v>1366</v>
+        <v>1363</v>
       </c>
       <c r="O216" s="4" t="s">
         <v>112</v>
@@ -13084,28 +13105,28 @@
         <v>216</v>
       </c>
       <c r="C217" s="5" t="s">
-        <v>1367</v>
+        <v>1364</v>
       </c>
       <c r="G217" s="5" t="s">
-        <v>1368</v>
+        <v>1365</v>
       </c>
       <c r="I217" s="5" t="s">
-        <v>1369</v>
+        <v>1366</v>
       </c>
       <c r="J217" s="5" t="s">
         <v>274</v>
       </c>
       <c r="K217" s="5" t="s">
-        <v>1370</v>
+        <v>1367</v>
       </c>
       <c r="L217" s="5" t="s">
         <v>827</v>
       </c>
       <c r="M217" s="5" t="s">
-        <v>1371</v>
+        <v>1368</v>
       </c>
       <c r="N217" s="5" t="s">
-        <v>1372</v>
+        <v>1369</v>
       </c>
       <c r="O217" s="4" t="s">
         <v>112</v>
@@ -13122,28 +13143,28 @@
         <v>217</v>
       </c>
       <c r="C218" s="5" t="s">
-        <v>1373</v>
+        <v>1370</v>
       </c>
       <c r="G218" s="5" t="s">
-        <v>1374</v>
+        <v>1371</v>
       </c>
       <c r="I218" s="5" t="s">
-        <v>1375</v>
+        <v>1372</v>
       </c>
       <c r="J218" s="5" t="s">
         <v>126</v>
       </c>
       <c r="K218" s="5" t="s">
-        <v>1376</v>
+        <v>1373</v>
       </c>
       <c r="L218" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M218" s="5" t="s">
-        <v>1377</v>
+        <v>1374</v>
       </c>
       <c r="N218" s="5" t="s">
-        <v>1378</v>
+        <v>1375</v>
       </c>
       <c r="O218" s="4" t="s">
         <v>837</v>
@@ -13157,31 +13178,31 @@
         <v>218</v>
       </c>
       <c r="C219" s="5" t="s">
-        <v>1379</v>
+        <v>1376</v>
       </c>
       <c r="G219" s="5" t="s">
-        <v>1380</v>
+        <v>1377</v>
       </c>
       <c r="I219" s="5" t="s">
-        <v>1381</v>
+        <v>1378</v>
       </c>
       <c r="J219" s="5" t="s">
         <v>580</v>
       </c>
       <c r="K219" s="5" t="s">
+        <v>1379</v>
+      </c>
+      <c r="L219" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M219" s="5" t="s">
+        <v>1380</v>
+      </c>
+      <c r="N219" s="5" t="s">
+        <v>1381</v>
+      </c>
+      <c r="O219" s="4" t="s">
         <v>1382</v>
-      </c>
-      <c r="L219" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M219" s="5" t="s">
-        <v>1383</v>
-      </c>
-      <c r="N219" s="5" t="s">
-        <v>1384</v>
-      </c>
-      <c r="O219" s="4" t="s">
-        <v>1385</v>
       </c>
     </row>
     <row r="220" spans="1:21">
@@ -13189,16 +13210,16 @@
         <v>219</v>
       </c>
       <c r="C220" s="5" t="s">
+        <v>1383</v>
+      </c>
+      <c r="G220" s="5" t="s">
+        <v>1384</v>
+      </c>
+      <c r="H220" s="3" t="s">
+        <v>1385</v>
+      </c>
+      <c r="I220" s="5" t="s">
         <v>1386</v>
-      </c>
-      <c r="G220" s="5" t="s">
-        <v>1387</v>
-      </c>
-      <c r="H220" s="3" t="s">
-        <v>1388</v>
-      </c>
-      <c r="I220" s="5" t="s">
-        <v>1389</v>
       </c>
       <c r="J220" s="5" t="s">
         <v>142</v>
@@ -13210,10 +13231,10 @@
         <v>47</v>
       </c>
       <c r="M220" s="5" t="s">
-        <v>1390</v>
+        <v>1387</v>
       </c>
       <c r="N220" s="5" t="s">
-        <v>1391</v>
+        <v>1388</v>
       </c>
       <c r="O220" s="4" t="s">
         <v>1050</v>
@@ -13224,25 +13245,25 @@
         <v>220</v>
       </c>
       <c r="C221" s="5" t="s">
-        <v>1392</v>
+        <v>1389</v>
       </c>
       <c r="G221" s="5" t="s">
-        <v>1393</v>
+        <v>1390</v>
       </c>
       <c r="I221" s="5" t="s">
-        <v>1394</v>
+        <v>1391</v>
       </c>
       <c r="J221" s="5" t="s">
         <v>60</v>
       </c>
       <c r="K221" s="5" t="s">
-        <v>1395</v>
+        <v>1392</v>
       </c>
       <c r="L221" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M221" s="5" t="s">
-        <v>1396</v>
+        <v>1393</v>
       </c>
       <c r="N221" s="5"/>
       <c r="O221" s="4" t="s">
@@ -13254,32 +13275,32 @@
         <v>221</v>
       </c>
       <c r="C222" s="5" t="s">
+        <v>1394</v>
+      </c>
+      <c r="G222" s="5" t="s">
+        <v>1395</v>
+      </c>
+      <c r="I222" s="5" t="s">
+        <v>1396</v>
+      </c>
+      <c r="J222" s="5" t="s">
         <v>1397</v>
       </c>
-      <c r="G222" s="5" t="s">
+      <c r="K222" s="5" t="s">
         <v>1398</v>
       </c>
-      <c r="I222" s="5" t="s">
+      <c r="L222" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M222" s="5" t="s">
         <v>1399</v>
-      </c>
-      <c r="J222" s="5" t="s">
-        <v>1400</v>
-      </c>
-      <c r="K222" s="5" t="s">
-        <v>1401</v>
-      </c>
-      <c r="L222" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M222" s="5" t="s">
-        <v>1402</v>
       </c>
       <c r="N222" s="5"/>
       <c r="O222" s="4" t="s">
-        <v>1403</v>
+        <v>1400</v>
       </c>
       <c r="P222" s="4" t="s">
-        <v>1404</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="223" spans="1:21">
@@ -13287,25 +13308,25 @@
         <v>222</v>
       </c>
       <c r="C223" s="5" t="s">
-        <v>1405</v>
+        <v>1402</v>
       </c>
       <c r="G223" s="5" t="s">
-        <v>1406</v>
+        <v>1403</v>
       </c>
       <c r="I223" s="5" t="s">
-        <v>1407</v>
+        <v>1404</v>
       </c>
       <c r="J223" s="5" t="s">
         <v>45</v>
       </c>
       <c r="K223" s="5" t="s">
-        <v>1408</v>
+        <v>1405</v>
       </c>
       <c r="L223" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M223" s="5" t="s">
-        <v>1409</v>
+        <v>1406</v>
       </c>
       <c r="N223" s="5"/>
       <c r="O223" s="4" t="s">
@@ -13317,10 +13338,10 @@
         <v>223</v>
       </c>
       <c r="C224" s="5" t="s">
-        <v>1410</v>
+        <v>1407</v>
       </c>
       <c r="G224" s="5" t="s">
-        <v>1411</v>
+        <v>1408</v>
       </c>
       <c r="I224" s="5" t="s">
         <v>199</v>
@@ -13329,16 +13350,16 @@
         <v>54</v>
       </c>
       <c r="K224" s="5" t="s">
-        <v>1412</v>
+        <v>1409</v>
       </c>
       <c r="L224" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M224" s="5" t="s">
-        <v>1413</v>
+        <v>1410</v>
       </c>
       <c r="N224" s="5" t="s">
-        <v>1414</v>
+        <v>1411</v>
       </c>
       <c r="O224" s="4" t="s">
         <v>78</v>
@@ -13349,24 +13370,24 @@
         <v>224</v>
       </c>
       <c r="C225" s="5" t="s">
-        <v>1415</v>
+        <v>1412</v>
       </c>
       <c r="G225" s="5" t="s">
-        <v>1416</v>
+        <v>1413</v>
       </c>
       <c r="I225" s="5" t="s">
-        <v>1417</v>
+        <v>1414</v>
       </c>
       <c r="J225" s="5"/>
       <c r="K225" s="5"/>
       <c r="L225" s="5" t="s">
-        <v>1418</v>
+        <v>1415</v>
       </c>
       <c r="M225" s="5" t="s">
-        <v>1419</v>
+        <v>1416</v>
       </c>
       <c r="N225" s="5" t="s">
-        <v>1420</v>
+        <v>1417</v>
       </c>
       <c r="O225" s="4" t="s">
         <v>78</v>
@@ -13377,28 +13398,28 @@
         <v>225</v>
       </c>
       <c r="C226" s="5" t="s">
-        <v>1421</v>
+        <v>1418</v>
       </c>
       <c r="G226" s="5" t="s">
-        <v>1422</v>
+        <v>1419</v>
       </c>
       <c r="I226" s="5" t="s">
-        <v>1423</v>
+        <v>1420</v>
       </c>
       <c r="J226" s="5" t="s">
         <v>239</v>
       </c>
       <c r="K226" s="5" t="s">
-        <v>1424</v>
+        <v>1421</v>
       </c>
       <c r="L226" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M226" s="5" t="s">
-        <v>1425</v>
+        <v>1422</v>
       </c>
       <c r="N226" s="5" t="s">
-        <v>1426</v>
+        <v>1423</v>
       </c>
       <c r="O226" s="4" t="s">
         <v>112</v>
@@ -13409,28 +13430,28 @@
         <v>226</v>
       </c>
       <c r="C227" s="5" t="s">
-        <v>1427</v>
+        <v>1424</v>
       </c>
       <c r="G227" s="5" t="s">
-        <v>1428</v>
+        <v>1425</v>
       </c>
       <c r="I227" s="5" t="s">
-        <v>1429</v>
+        <v>1426</v>
       </c>
       <c r="J227" s="5" t="s">
         <v>324</v>
       </c>
       <c r="K227" s="5" t="s">
-        <v>1430</v>
+        <v>1427</v>
       </c>
       <c r="L227" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M227" s="5" t="s">
-        <v>1431</v>
+        <v>1428</v>
       </c>
       <c r="N227" s="5" t="s">
-        <v>1432</v>
+        <v>1429</v>
       </c>
       <c r="O227" s="4" t="s">
         <v>112</v>
@@ -13441,28 +13462,28 @@
         <v>227</v>
       </c>
       <c r="C228" s="5" t="s">
-        <v>1433</v>
+        <v>1430</v>
       </c>
       <c r="G228" s="5" t="s">
-        <v>1434</v>
+        <v>1431</v>
       </c>
       <c r="I228" s="5" t="s">
-        <v>1435</v>
+        <v>1432</v>
       </c>
       <c r="J228" s="5" t="s">
         <v>60</v>
       </c>
       <c r="K228" s="5" t="s">
-        <v>1436</v>
+        <v>1433</v>
       </c>
       <c r="L228" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M228" s="5" t="s">
-        <v>1437</v>
+        <v>1434</v>
       </c>
       <c r="N228" s="5" t="s">
-        <v>1438</v>
+        <v>1435</v>
       </c>
       <c r="O228" s="4" t="s">
         <v>170</v>
@@ -13473,25 +13494,25 @@
         <v>228</v>
       </c>
       <c r="C229" s="5" t="s">
-        <v>1439</v>
+        <v>1436</v>
       </c>
       <c r="G229" s="5" t="s">
-        <v>1440</v>
+        <v>1437</v>
       </c>
       <c r="I229" s="5" t="s">
-        <v>1441</v>
+        <v>1438</v>
       </c>
       <c r="J229" s="5" t="s">
         <v>219</v>
       </c>
       <c r="K229" s="5" t="s">
-        <v>1442</v>
+        <v>1439</v>
       </c>
       <c r="L229" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M229" s="5" t="s">
-        <v>1443</v>
+        <v>1440</v>
       </c>
       <c r="N229" s="5"/>
       <c r="O229" s="4" t="s">
@@ -13503,28 +13524,28 @@
         <v>229</v>
       </c>
       <c r="C230" s="5" t="s">
-        <v>1444</v>
+        <v>1441</v>
       </c>
       <c r="G230" s="5" t="s">
-        <v>1445</v>
+        <v>1442</v>
       </c>
       <c r="I230" s="5" t="s">
-        <v>1446</v>
+        <v>1443</v>
       </c>
       <c r="J230" s="5" t="s">
         <v>299</v>
       </c>
       <c r="K230" s="5" t="s">
-        <v>1447</v>
+        <v>1444</v>
       </c>
       <c r="L230" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M230" s="5" t="s">
-        <v>1448</v>
+        <v>1445</v>
       </c>
       <c r="N230" s="5" t="s">
-        <v>1449</v>
+        <v>1446</v>
       </c>
       <c r="O230" s="4" t="s">
         <v>170</v>
@@ -13535,28 +13556,28 @@
         <v>230</v>
       </c>
       <c r="C231" s="5" t="s">
-        <v>1450</v>
+        <v>1447</v>
       </c>
       <c r="G231" s="5" t="s">
-        <v>1451</v>
+        <v>1448</v>
       </c>
       <c r="I231" s="5" t="s">
-        <v>1452</v>
+        <v>1449</v>
       </c>
       <c r="J231" s="5" t="s">
         <v>226</v>
       </c>
       <c r="K231" s="5" t="s">
-        <v>1453</v>
+        <v>1450</v>
       </c>
       <c r="L231" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M231" s="5" t="s">
-        <v>1454</v>
+        <v>1451</v>
       </c>
       <c r="N231" s="5" t="s">
-        <v>1455</v>
+        <v>1452</v>
       </c>
       <c r="O231" s="4" t="s">
         <v>170</v>
@@ -13567,28 +13588,28 @@
         <v>231</v>
       </c>
       <c r="C232" s="5" t="s">
-        <v>1456</v>
+        <v>1453</v>
       </c>
       <c r="G232" s="5" t="s">
-        <v>1457</v>
+        <v>1454</v>
       </c>
       <c r="I232" s="5" t="s">
-        <v>1458</v>
+        <v>1455</v>
       </c>
       <c r="J232" s="5" t="s">
         <v>783</v>
       </c>
       <c r="K232" s="5" t="s">
-        <v>1459</v>
+        <v>1456</v>
       </c>
       <c r="L232" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M232" s="5" t="s">
-        <v>1460</v>
+        <v>1457</v>
       </c>
       <c r="N232" s="5" t="s">
-        <v>1461</v>
+        <v>1458</v>
       </c>
       <c r="O232" s="4" t="s">
         <v>170</v>
@@ -13599,10 +13620,10 @@
         <v>232</v>
       </c>
       <c r="C233" s="5" t="s">
-        <v>1462</v>
+        <v>1459</v>
       </c>
       <c r="G233" s="5" t="s">
-        <v>1463</v>
+        <v>1460</v>
       </c>
       <c r="I233" s="5" t="s">
         <v>361</v>
@@ -13611,16 +13632,16 @@
         <v>299</v>
       </c>
       <c r="K233" s="5" t="s">
-        <v>1464</v>
+        <v>1461</v>
       </c>
       <c r="L233" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M233" s="5" t="s">
-        <v>1465</v>
+        <v>1462</v>
       </c>
       <c r="N233" s="5" t="s">
-        <v>1466</v>
+        <v>1463</v>
       </c>
       <c r="O233" s="4" t="s">
         <v>112</v>
@@ -13631,13 +13652,13 @@
         <v>233</v>
       </c>
       <c r="C234" s="5" t="s">
-        <v>1467</v>
+        <v>1464</v>
       </c>
       <c r="G234" s="5" t="s">
-        <v>1468</v>
+        <v>1465</v>
       </c>
       <c r="H234" s="3" t="s">
-        <v>1469</v>
+        <v>1466</v>
       </c>
       <c r="I234" s="5" t="s">
         <v>856</v>
@@ -13646,16 +13667,16 @@
         <v>67</v>
       </c>
       <c r="K234" s="5" t="s">
-        <v>1470</v>
+        <v>1467</v>
       </c>
       <c r="L234" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M234" s="5" t="s">
-        <v>1471</v>
+        <v>1468</v>
       </c>
       <c r="N234" s="5" t="s">
-        <v>1472</v>
+        <v>1469</v>
       </c>
       <c r="O234" s="4" t="s">
         <v>170</v>
@@ -13666,10 +13687,10 @@
         <v>234</v>
       </c>
       <c r="C235" s="5" t="s">
-        <v>1473</v>
+        <v>1470</v>
       </c>
       <c r="G235" s="5" t="s">
-        <v>1474</v>
+        <v>1471</v>
       </c>
       <c r="I235" s="5" t="s">
         <v>218</v>
@@ -13678,16 +13699,16 @@
         <v>580</v>
       </c>
       <c r="K235" s="5" t="s">
-        <v>1475</v>
+        <v>1472</v>
       </c>
       <c r="L235" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M235" s="5" t="s">
-        <v>1476</v>
+        <v>1473</v>
       </c>
       <c r="N235" s="5" t="s">
-        <v>1477</v>
+        <v>1474</v>
       </c>
       <c r="O235" s="4" t="s">
         <v>49</v>
@@ -13698,10 +13719,10 @@
         <v>235</v>
       </c>
       <c r="C236" s="5" t="s">
-        <v>1478</v>
+        <v>1475</v>
       </c>
       <c r="G236" s="5" t="s">
-        <v>1479</v>
+        <v>1476</v>
       </c>
       <c r="I236" s="5" t="s">
         <v>820</v>
@@ -13710,16 +13731,16 @@
         <v>126</v>
       </c>
       <c r="K236" s="5" t="s">
-        <v>1480</v>
+        <v>1477</v>
       </c>
       <c r="L236" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M236" s="5" t="s">
-        <v>1481</v>
+        <v>1478</v>
       </c>
       <c r="N236" s="5" t="s">
-        <v>1482</v>
+        <v>1479</v>
       </c>
       <c r="O236" s="4" t="s">
         <v>49</v>
@@ -13736,26 +13757,26 @@
         <v>236</v>
       </c>
       <c r="C237" s="5" t="s">
-        <v>1483</v>
+        <v>1480</v>
       </c>
       <c r="G237" s="5" t="s">
-        <v>1484</v>
+        <v>1481</v>
       </c>
       <c r="I237" s="5" t="s">
-        <v>1485</v>
+        <v>1482</v>
       </c>
       <c r="J237" s="5" t="s">
         <v>482</v>
       </c>
       <c r="K237" s="5" t="s">
-        <v>1486</v>
+        <v>1483</v>
       </c>
       <c r="L237" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M237" s="5"/>
       <c r="N237" s="5" t="s">
-        <v>1487</v>
+        <v>1484</v>
       </c>
       <c r="O237" s="4" t="s">
         <v>170</v>
@@ -13766,10 +13787,10 @@
         <v>237</v>
       </c>
       <c r="C238" s="5" t="s">
-        <v>1488</v>
+        <v>1485</v>
       </c>
       <c r="G238" s="5" t="s">
-        <v>1489</v>
+        <v>1486</v>
       </c>
       <c r="I238" s="5" t="s">
         <v>792</v>
@@ -13778,16 +13799,16 @@
         <v>464</v>
       </c>
       <c r="K238" s="5" t="s">
-        <v>1490</v>
+        <v>1487</v>
       </c>
       <c r="L238" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M238" s="5" t="s">
-        <v>1491</v>
+        <v>1488</v>
       </c>
       <c r="N238" s="5" t="s">
-        <v>1492</v>
+        <v>1489</v>
       </c>
       <c r="O238" s="4" t="s">
         <v>78</v>
@@ -13801,10 +13822,10 @@
         <v>238</v>
       </c>
       <c r="C239" s="5" t="s">
-        <v>1493</v>
+        <v>1490</v>
       </c>
       <c r="G239" s="5" t="s">
-        <v>1494</v>
+        <v>1491</v>
       </c>
       <c r="I239" s="5" t="s">
         <v>934</v>
@@ -13813,16 +13834,16 @@
         <v>299</v>
       </c>
       <c r="K239" s="5" t="s">
-        <v>1495</v>
+        <v>1492</v>
       </c>
       <c r="L239" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M239" s="5" t="s">
-        <v>1496</v>
+        <v>1493</v>
       </c>
       <c r="N239" s="5" t="s">
-        <v>1497</v>
+        <v>1494</v>
       </c>
       <c r="O239" s="4" t="s">
         <v>78</v>
@@ -13833,28 +13854,28 @@
         <v>239</v>
       </c>
       <c r="C240" s="5" t="s">
+        <v>1495</v>
+      </c>
+      <c r="G240" s="5" t="s">
+        <v>1496</v>
+      </c>
+      <c r="I240" s="5" t="s">
+        <v>1497</v>
+      </c>
+      <c r="J240" s="5" t="s">
         <v>1498</v>
       </c>
-      <c r="G240" s="5" t="s">
+      <c r="K240" s="5" t="s">
         <v>1499</v>
       </c>
-      <c r="I240" s="5" t="s">
+      <c r="L240" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M240" s="5" t="s">
         <v>1500</v>
       </c>
-      <c r="J240" s="5" t="s">
+      <c r="N240" s="5" t="s">
         <v>1501</v>
-      </c>
-      <c r="K240" s="5" t="s">
-        <v>1502</v>
-      </c>
-      <c r="L240" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M240" s="5" t="s">
-        <v>1503</v>
-      </c>
-      <c r="N240" s="5" t="s">
-        <v>1504</v>
       </c>
       <c r="O240" s="4" t="s">
         <v>78</v>
@@ -13869,28 +13890,28 @@
       </c>
       <c r="B241" s="3"/>
       <c r="C241" s="7" t="s">
-        <v>1505</v>
+        <v>1502</v>
       </c>
       <c r="G241" s="7" t="s">
-        <v>1506</v>
+        <v>1503</v>
       </c>
       <c r="I241" s="7" t="s">
-        <v>1485</v>
+        <v>1482</v>
       </c>
       <c r="J241" s="7" t="s">
         <v>219</v>
       </c>
       <c r="K241" s="7" t="s">
-        <v>1507</v>
+        <v>1504</v>
       </c>
       <c r="L241" s="7" t="s">
         <v>47</v>
       </c>
       <c r="M241" s="7" t="s">
-        <v>1508</v>
+        <v>1505</v>
       </c>
       <c r="N241" s="7" t="s">
-        <v>1505</v>
+        <v>1502</v>
       </c>
       <c r="O241" s="10" t="s">
         <v>112</v>
@@ -13907,34 +13928,34 @@
         <v>241</v>
       </c>
       <c r="C242" s="5" t="s">
+        <v>1506</v>
+      </c>
+      <c r="G242" s="5" t="s">
+        <v>1507</v>
+      </c>
+      <c r="H242" s="3" t="s">
+        <v>1508</v>
+      </c>
+      <c r="I242" s="5" t="s">
         <v>1509</v>
-      </c>
-      <c r="G242" s="5" t="s">
-        <v>1510</v>
-      </c>
-      <c r="H242" s="3" t="s">
-        <v>1511</v>
-      </c>
-      <c r="I242" s="5" t="s">
-        <v>1512</v>
       </c>
       <c r="J242" s="5" t="s">
         <v>54</v>
       </c>
       <c r="K242" s="5" t="s">
-        <v>1513</v>
+        <v>1510</v>
       </c>
       <c r="L242" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M242" s="5" t="s">
-        <v>1514</v>
+        <v>1511</v>
       </c>
       <c r="N242" s="5" t="s">
-        <v>1515</v>
+        <v>1512</v>
       </c>
       <c r="O242" s="4" t="s">
-        <v>1356</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="243" spans="1:21">
@@ -13942,28 +13963,28 @@
         <v>242</v>
       </c>
       <c r="C243" s="5" t="s">
+        <v>1513</v>
+      </c>
+      <c r="G243" s="5" t="s">
+        <v>1514</v>
+      </c>
+      <c r="I243" s="5" t="s">
+        <v>1515</v>
+      </c>
+      <c r="J243" s="5" t="s">
         <v>1516</v>
       </c>
-      <c r="G243" s="5" t="s">
+      <c r="K243" s="5" t="s">
         <v>1517</v>
       </c>
-      <c r="I243" s="5" t="s">
+      <c r="L243" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M243" s="5" t="s">
         <v>1518</v>
       </c>
-      <c r="J243" s="5" t="s">
+      <c r="N243" s="5" t="s">
         <v>1519</v>
-      </c>
-      <c r="K243" s="5" t="s">
-        <v>1520</v>
-      </c>
-      <c r="L243" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M243" s="5" t="s">
-        <v>1521</v>
-      </c>
-      <c r="N243" s="5" t="s">
-        <v>1522</v>
       </c>
       <c r="O243" s="4" t="s">
         <v>170</v>
@@ -13974,10 +13995,10 @@
         <v>243</v>
       </c>
       <c r="C244" s="5" t="s">
-        <v>1523</v>
+        <v>1520</v>
       </c>
       <c r="G244" s="5" t="s">
-        <v>1524</v>
+        <v>1521</v>
       </c>
       <c r="I244" s="5" t="s">
         <v>856</v>
@@ -13986,13 +14007,13 @@
         <v>67</v>
       </c>
       <c r="K244" s="5" t="s">
-        <v>1525</v>
+        <v>1522</v>
       </c>
       <c r="L244" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M244" s="5" t="s">
-        <v>1526</v>
+        <v>1523</v>
       </c>
       <c r="N244" s="5"/>
       <c r="O244" s="4" t="s">
@@ -14004,28 +14025,28 @@
         <v>244</v>
       </c>
       <c r="C245" s="5" t="s">
-        <v>1527</v>
+        <v>1524</v>
       </c>
       <c r="G245" s="5" t="s">
-        <v>1528</v>
+        <v>1525</v>
       </c>
       <c r="I245" s="5" t="s">
-        <v>1529</v>
+        <v>1526</v>
       </c>
       <c r="J245" s="5" t="s">
         <v>627</v>
       </c>
       <c r="K245" s="5" t="s">
-        <v>1530</v>
+        <v>1527</v>
       </c>
       <c r="L245" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M245" s="5" t="s">
-        <v>1531</v>
+        <v>1528</v>
       </c>
       <c r="N245" s="5" t="s">
-        <v>1532</v>
+        <v>1529</v>
       </c>
       <c r="O245" s="4" t="s">
         <v>78</v>
@@ -14036,28 +14057,28 @@
         <v>245</v>
       </c>
       <c r="C246" s="5" t="s">
-        <v>1533</v>
+        <v>1530</v>
       </c>
       <c r="G246" s="5" t="s">
-        <v>1534</v>
+        <v>1531</v>
       </c>
       <c r="I246" s="5" t="s">
-        <v>1535</v>
+        <v>1532</v>
       </c>
       <c r="J246" s="5" t="s">
         <v>627</v>
       </c>
       <c r="K246" s="5" t="s">
-        <v>1536</v>
+        <v>1533</v>
       </c>
       <c r="L246" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M246" s="5" t="s">
-        <v>1537</v>
+        <v>1534</v>
       </c>
       <c r="N246" s="5" t="s">
-        <v>1538</v>
+        <v>1535</v>
       </c>
       <c r="O246" s="4" t="s">
         <v>170</v>
@@ -14068,28 +14089,28 @@
         <v>246</v>
       </c>
       <c r="C247" s="5" t="s">
-        <v>1539</v>
+        <v>1536</v>
       </c>
       <c r="G247" s="5" t="s">
-        <v>1540</v>
+        <v>1537</v>
       </c>
       <c r="I247" s="5" t="s">
-        <v>1535</v>
+        <v>1532</v>
       </c>
       <c r="J247" s="5" t="s">
         <v>60</v>
       </c>
       <c r="K247" s="5" t="s">
-        <v>1541</v>
+        <v>1538</v>
       </c>
       <c r="L247" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M247" s="5" t="s">
-        <v>1542</v>
+        <v>1539</v>
       </c>
       <c r="N247" s="5" t="s">
-        <v>1543</v>
+        <v>1540</v>
       </c>
       <c r="O247" s="4" t="s">
         <v>170</v>
@@ -14100,28 +14121,28 @@
         <v>247</v>
       </c>
       <c r="C248" s="5" t="s">
-        <v>1544</v>
+        <v>1541</v>
       </c>
       <c r="G248" s="5" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
       <c r="I248" s="5" t="s">
-        <v>1546</v>
+        <v>1543</v>
       </c>
       <c r="J248" s="5" t="s">
         <v>299</v>
       </c>
       <c r="K248" s="5" t="s">
-        <v>1547</v>
+        <v>1544</v>
       </c>
       <c r="L248" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M248" s="5" t="s">
-        <v>1548</v>
+        <v>1545</v>
       </c>
       <c r="N248" s="5" t="s">
-        <v>1549</v>
+        <v>1546</v>
       </c>
       <c r="O248" s="4" t="s">
         <v>112</v>
@@ -14132,25 +14153,25 @@
         <v>248</v>
       </c>
       <c r="C249" s="5" t="s">
-        <v>1550</v>
+        <v>1547</v>
       </c>
       <c r="G249" s="5" t="s">
-        <v>1551</v>
+        <v>1548</v>
       </c>
       <c r="I249" s="5" t="s">
-        <v>1552</v>
+        <v>1549</v>
       </c>
       <c r="J249" s="5" t="s">
         <v>126</v>
       </c>
       <c r="K249" s="5" t="s">
-        <v>1553</v>
+        <v>1550</v>
       </c>
       <c r="L249" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M249" s="5" t="s">
-        <v>1554</v>
+        <v>1551</v>
       </c>
       <c r="N249" s="5"/>
       <c r="O249" s="4" t="s">
@@ -14162,10 +14183,10 @@
         <v>249</v>
       </c>
       <c r="C250" s="5" t="s">
-        <v>1555</v>
+        <v>1552</v>
       </c>
       <c r="G250" s="5" t="s">
-        <v>1556</v>
+        <v>1553</v>
       </c>
       <c r="I250" s="5" t="s">
         <v>856</v>
@@ -14180,10 +14201,10 @@
         <v>47</v>
       </c>
       <c r="M250" s="5" t="s">
-        <v>1557</v>
+        <v>1554</v>
       </c>
       <c r="N250" s="5" t="s">
-        <v>1558</v>
+        <v>1555</v>
       </c>
       <c r="O250" s="4" t="s">
         <v>112</v>
@@ -14197,25 +14218,25 @@
         <v>250</v>
       </c>
       <c r="C251" s="5" t="s">
-        <v>1559</v>
+        <v>1556</v>
       </c>
       <c r="G251" s="5" t="s">
-        <v>1560</v>
+        <v>1557</v>
       </c>
       <c r="I251" s="5" t="s">
-        <v>1561</v>
+        <v>1558</v>
       </c>
       <c r="J251" s="5" t="s">
         <v>54</v>
       </c>
       <c r="K251" s="5" t="s">
-        <v>1562</v>
+        <v>1559</v>
       </c>
       <c r="L251" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M251" s="5" t="s">
-        <v>1563</v>
+        <v>1560</v>
       </c>
       <c r="N251" s="5"/>
       <c r="O251" s="4" t="s">
@@ -14227,28 +14248,28 @@
         <v>251</v>
       </c>
       <c r="C252" s="5" t="s">
-        <v>1564</v>
+        <v>1561</v>
       </c>
       <c r="G252" s="5" t="s">
-        <v>1565</v>
+        <v>1562</v>
       </c>
       <c r="I252" s="5" t="s">
-        <v>1566</v>
+        <v>1563</v>
       </c>
       <c r="J252" s="5" t="s">
         <v>45</v>
       </c>
       <c r="K252" s="5" t="s">
-        <v>1567</v>
+        <v>1564</v>
       </c>
       <c r="L252" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M252" s="5" t="s">
-        <v>1568</v>
+        <v>1565</v>
       </c>
       <c r="N252" s="5" t="s">
-        <v>1569</v>
+        <v>1566</v>
       </c>
       <c r="O252" s="4" t="s">
         <v>112</v>
@@ -14266,29 +14287,29 @@
       </c>
       <c r="B253" s="3"/>
       <c r="C253" s="7" t="s">
-        <v>1570</v>
+        <v>1567</v>
       </c>
       <c r="G253" s="7" t="s">
-        <v>1571</v>
+        <v>1568</v>
       </c>
       <c r="I253" s="7" t="s">
-        <v>1572</v>
+        <v>1569</v>
       </c>
       <c r="J253" s="7" t="s">
         <v>45</v>
       </c>
       <c r="K253" s="7" t="s">
-        <v>1573</v>
+        <v>1570</v>
       </c>
       <c r="L253" s="7" t="s">
         <v>47</v>
       </c>
       <c r="M253" s="7" t="s">
-        <v>1574</v>
+        <v>1571</v>
       </c>
       <c r="N253" s="7"/>
       <c r="O253" s="10" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
       <c r="P253" s="10"/>
       <c r="Q253" s="10"/>
@@ -14302,31 +14323,31 @@
         <v>253</v>
       </c>
       <c r="C254" s="5" t="s">
-        <v>1575</v>
+        <v>1572</v>
       </c>
       <c r="G254" s="5" t="s">
-        <v>1576</v>
+        <v>1573</v>
       </c>
       <c r="I254" s="5" t="s">
-        <v>1577</v>
+        <v>1574</v>
       </c>
       <c r="J254" s="5" t="s">
         <v>226</v>
       </c>
       <c r="K254" s="5" t="s">
-        <v>1578</v>
+        <v>1575</v>
       </c>
       <c r="L254" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M254" s="5" t="s">
-        <v>1579</v>
+        <v>1576</v>
       </c>
       <c r="N254" s="5" t="s">
-        <v>1580</v>
+        <v>1577</v>
       </c>
       <c r="O254" s="4" t="s">
-        <v>1385</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="255" spans="1:21">
@@ -14334,10 +14355,10 @@
         <v>254</v>
       </c>
       <c r="C255" s="5" t="s">
-        <v>1581</v>
+        <v>1578</v>
       </c>
       <c r="G255" s="5" t="s">
-        <v>1582</v>
+        <v>1579</v>
       </c>
       <c r="I255" s="5" t="s">
         <v>387</v>
@@ -14346,19 +14367,19 @@
         <v>226</v>
       </c>
       <c r="K255" s="5" t="s">
-        <v>1583</v>
+        <v>1580</v>
       </c>
       <c r="L255" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M255" s="5" t="s">
-        <v>1584</v>
+        <v>1581</v>
       </c>
       <c r="N255" s="5" t="s">
-        <v>1585</v>
+        <v>1582</v>
       </c>
       <c r="O255" s="4" t="s">
-        <v>1385</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="256" spans="1:21">
@@ -14366,10 +14387,10 @@
         <v>255</v>
       </c>
       <c r="C256" s="5" t="s">
-        <v>1586</v>
+        <v>1583</v>
       </c>
       <c r="G256" s="5" t="s">
-        <v>1587</v>
+        <v>1584</v>
       </c>
       <c r="I256" s="5" t="s">
         <v>652</v>
@@ -14378,19 +14399,19 @@
         <v>54</v>
       </c>
       <c r="K256" s="5" t="s">
-        <v>1588</v>
+        <v>1585</v>
       </c>
       <c r="L256" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M256" s="5" t="s">
-        <v>1589</v>
+        <v>1586</v>
       </c>
       <c r="N256" s="5" t="s">
-        <v>1590</v>
+        <v>1587</v>
       </c>
       <c r="O256" s="4" t="s">
-        <v>1277</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="257" spans="1:16">
@@ -14398,10 +14419,10 @@
         <v>256</v>
       </c>
       <c r="C257" s="5" t="s">
-        <v>1591</v>
+        <v>1588</v>
       </c>
       <c r="G257" s="5" t="s">
-        <v>1592</v>
+        <v>1589</v>
       </c>
       <c r="I257" s="5" t="s">
         <v>798</v>
@@ -14410,16 +14431,16 @@
         <v>783</v>
       </c>
       <c r="K257" s="5" t="s">
-        <v>1593</v>
+        <v>1590</v>
       </c>
       <c r="L257" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M257" s="5" t="s">
-        <v>1594</v>
+        <v>1591</v>
       </c>
       <c r="N257" s="5" t="s">
-        <v>1595</v>
+        <v>1592</v>
       </c>
       <c r="O257" s="4" t="s">
         <v>49</v>
@@ -14430,25 +14451,25 @@
         <v>257</v>
       </c>
       <c r="C258" s="5" t="s">
-        <v>1596</v>
+        <v>1593</v>
       </c>
       <c r="G258" s="5" t="s">
-        <v>1597</v>
+        <v>1594</v>
       </c>
       <c r="I258" s="5" t="s">
-        <v>1598</v>
+        <v>1595</v>
       </c>
       <c r="J258" s="5" t="s">
         <v>247</v>
       </c>
       <c r="K258" s="5" t="s">
-        <v>1599</v>
+        <v>1596</v>
       </c>
       <c r="L258" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M258" s="5" t="s">
-        <v>1600</v>
+        <v>1597</v>
       </c>
       <c r="N258" s="5"/>
       <c r="O258" s="4" t="s">
@@ -14460,28 +14481,28 @@
         <v>258</v>
       </c>
       <c r="C259" s="5" t="s">
-        <v>1601</v>
+        <v>1598</v>
       </c>
       <c r="G259" s="5" t="s">
-        <v>1602</v>
+        <v>1599</v>
       </c>
       <c r="I259" s="5" t="s">
-        <v>1429</v>
+        <v>1426</v>
       </c>
       <c r="J259" s="5" t="s">
         <v>324</v>
       </c>
       <c r="K259" s="5" t="s">
-        <v>1603</v>
+        <v>1600</v>
       </c>
       <c r="L259" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M259" s="5" t="s">
-        <v>1604</v>
+        <v>1601</v>
       </c>
       <c r="N259" s="5" t="s">
-        <v>1605</v>
+        <v>1602</v>
       </c>
       <c r="O259" s="4" t="s">
         <v>112</v>
@@ -14492,28 +14513,28 @@
         <v>259</v>
       </c>
       <c r="C260" s="5" t="s">
-        <v>1606</v>
+        <v>1603</v>
       </c>
       <c r="G260" s="5" t="s">
-        <v>1607</v>
+        <v>1604</v>
       </c>
       <c r="I260" s="5" t="s">
-        <v>1608</v>
+        <v>1605</v>
       </c>
       <c r="J260" s="5" t="s">
         <v>299</v>
       </c>
       <c r="K260" s="5" t="s">
-        <v>1609</v>
+        <v>1606</v>
       </c>
       <c r="L260" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M260" s="5" t="s">
-        <v>1610</v>
+        <v>1607</v>
       </c>
       <c r="N260" s="5" t="s">
-        <v>1611</v>
+        <v>1608</v>
       </c>
       <c r="O260" s="4" t="s">
         <v>112</v>
@@ -14524,25 +14545,25 @@
         <v>260</v>
       </c>
       <c r="C261" s="5" t="s">
-        <v>1612</v>
+        <v>1609</v>
       </c>
       <c r="G261" s="5" t="s">
-        <v>1613</v>
+        <v>1610</v>
       </c>
       <c r="I261" s="5" t="s">
-        <v>1614</v>
+        <v>1611</v>
       </c>
       <c r="J261" s="5" t="s">
         <v>299</v>
       </c>
       <c r="K261" s="5" t="s">
-        <v>1615</v>
+        <v>1612</v>
       </c>
       <c r="L261" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M261" s="5" t="s">
-        <v>1616</v>
+        <v>1613</v>
       </c>
       <c r="N261" s="5"/>
       <c r="O261" s="4" t="s">
@@ -14554,31 +14575,31 @@
         <v>261</v>
       </c>
       <c r="C262" s="5" t="s">
+        <v>1614</v>
+      </c>
+      <c r="G262" s="5" t="s">
+        <v>1615</v>
+      </c>
+      <c r="H262" s="3" t="s">
+        <v>1616</v>
+      </c>
+      <c r="I262" s="5" t="s">
+        <v>1515</v>
+      </c>
+      <c r="J262" s="5" t="s">
+        <v>1516</v>
+      </c>
+      <c r="K262" s="5" t="s">
         <v>1617</v>
       </c>
-      <c r="G262" s="5" t="s">
+      <c r="L262" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="M262" s="5" t="s">
         <v>1618</v>
       </c>
-      <c r="H262" s="3" t="s">
+      <c r="N262" s="5" t="s">
         <v>1619</v>
-      </c>
-      <c r="I262" s="5" t="s">
-        <v>1518</v>
-      </c>
-      <c r="J262" s="5" t="s">
-        <v>1519</v>
-      </c>
-      <c r="K262" s="5" t="s">
-        <v>1620</v>
-      </c>
-      <c r="L262" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="M262" s="5" t="s">
-        <v>1621</v>
-      </c>
-      <c r="N262" s="5" t="s">
-        <v>1622</v>
       </c>
       <c r="O262" s="4" t="s">
         <v>49</v>
@@ -14592,38 +14613,38 @@
         <v>262</v>
       </c>
       <c r="C263" s="5" t="s">
-        <v>1623</v>
+        <v>1620</v>
       </c>
       <c r="G263" s="5" t="s">
-        <v>1624</v>
+        <v>1621</v>
       </c>
       <c r="I263" s="5" t="s">
-        <v>1625</v>
+        <v>1622</v>
       </c>
       <c r="J263" s="5" t="s">
         <v>324</v>
       </c>
       <c r="K263" s="5" t="s">
-        <v>1626</v>
+        <v>1623</v>
       </c>
       <c r="L263" s="5" t="s">
         <v>47</v>
       </c>
       <c r="M263" s="5" t="s">
-        <v>1627</v>
+        <v>1624</v>
       </c>
       <c r="N263" s="5" t="s">
-        <v>1628</v>
+        <v>1625</v>
       </c>
       <c r="O263" s="4" t="s">
         <v>112</v>
       </c>
       <c r="P263" s="17" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AT1" xr:uid="{30F676E1-FBA3-424A-825B-7953DA4AF81C}"/>
+  <autoFilter ref="A1:AT263" xr:uid="{30F676E1-FBA3-424A-825B-7953DA4AF81C}"/>
   <hyperlinks>
     <hyperlink ref="N5" r:id="rId1" xr:uid="{A6B7692D-78AB-4552-8414-9ADC25CB65ED}"/>
   </hyperlinks>

</xml_diff>